<commit_message>
Update Project706_J. A. Long(2006).xlsx
</commit_message>
<xml_diff>
--- a/Project706_J. A. Long(2006).xlsx
+++ b/Project706_J. A. Long(2006).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjjg18\GitHub\neotrans\matrices\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/926c5b3b47b66c00/Documents/GitHub/matrices/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{253FBD24-E801-4C86-BB4F-9B1A3F3FF0B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16455" yWindow="3120" windowWidth="15945" windowHeight="18375" xr2:uid="{78ADB668-0A1D-7E4D-9DAF-AEFEFC7B5128}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{78ADB668-0A1D-7E4D-9DAF-AEFEFC7B5128}"/>
   </bookViews>
   <sheets>
     <sheet name="Project 706" sheetId="2" r:id="rId1"/>
@@ -480,6 +480,7 @@
       <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -876,13 +877,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2295819D-64F8-2241-8706-9DDF2FCC4E78}">
   <dimension ref="A1:C115"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="83.375" customWidth="1"/>
-    <col min="2" max="3" width="21.875" customWidth="1"/>
+    <col min="1" max="1" width="83.33203125" customWidth="1"/>
+    <col min="2" max="3" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -893,7 +894,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>122</v>
       </c>
@@ -904,7 +905,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -915,7 +916,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -926,7 +927,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -937,7 +938,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -948,7 +949,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -959,7 +960,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -970,7 +971,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -981,7 +982,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -992,7 +993,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1001,7 +1002,7 @@
       </c>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1012,7 +1013,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1023,7 +1024,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1034,7 +1035,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1043,7 +1044,7 @@
       </c>
       <c r="C15" s="2"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -1051,7 +1052,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1062,7 +1063,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1073,7 +1074,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1084,7 +1085,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1095,7 +1096,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1106,7 +1107,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1117,7 +1118,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1128,7 +1129,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1139,7 +1140,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1150,7 +1151,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1161,7 +1162,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1172,7 +1173,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1183,7 +1184,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -1194,7 +1195,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1203,7 +1204,7 @@
       </c>
       <c r="C30" s="1"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1214,7 +1215,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1225,7 +1226,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1236,7 +1237,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1247,7 +1248,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1258,7 +1259,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1267,7 +1268,7 @@
       </c>
       <c r="C36" s="1"/>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1278,7 +1279,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1289,7 +1290,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1300,7 +1301,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1311,7 +1312,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1322,7 +1323,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1333,7 +1334,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -1344,7 +1345,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -1355,7 +1356,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -1366,7 +1367,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -1377,7 +1378,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -1388,7 +1389,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -1399,7 +1400,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -1410,7 +1411,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>54</v>
       </c>
@@ -1421,7 +1422,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -1432,7 +1433,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>56</v>
       </c>
@@ -1443,7 +1444,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>57</v>
       </c>
@@ -1454,7 +1455,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>58</v>
       </c>
@@ -1465,7 +1466,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>59</v>
       </c>
@@ -1476,7 +1477,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>60</v>
       </c>
@@ -1487,7 +1488,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>61</v>
       </c>
@@ -1498,7 +1499,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>62</v>
       </c>
@@ -1509,7 +1510,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>63</v>
       </c>
@@ -1520,7 +1521,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
         <v>64</v>
       </c>
@@ -1531,7 +1532,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
         <v>65</v>
       </c>
@@ -1542,7 +1543,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
         <v>66</v>
       </c>
@@ -1553,7 +1554,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>67</v>
       </c>
@@ -1564,7 +1565,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -1575,7 +1576,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
         <v>69</v>
       </c>
@@ -1586,7 +1587,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
         <v>70</v>
       </c>
@@ -1597,7 +1598,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>71</v>
       </c>
@@ -1608,7 +1609,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
         <v>72</v>
       </c>
@@ -1619,7 +1620,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
         <v>73</v>
       </c>
@@ -1630,7 +1631,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
         <v>74</v>
       </c>
@@ -1641,7 +1642,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
         <v>75</v>
       </c>
@@ -1652,7 +1653,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
         <v>76</v>
       </c>
@@ -1663,7 +1664,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>77</v>
       </c>
@@ -1674,7 +1675,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
         <v>78</v>
       </c>
@@ -1685,7 +1686,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
         <v>79</v>
       </c>
@@ -1696,7 +1697,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>80</v>
       </c>
@@ -1707,7 +1708,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
         <v>81</v>
       </c>
@@ -1718,7 +1719,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
         <v>82</v>
       </c>
@@ -1729,7 +1730,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
         <v>83</v>
       </c>
@@ -1738,7 +1739,7 @@
       </c>
       <c r="C79" s="1"/>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>84</v>
       </c>
@@ -1749,7 +1750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>85</v>
       </c>
@@ -1760,7 +1761,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>86</v>
       </c>
@@ -1771,7 +1772,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
         <v>87</v>
       </c>
@@ -1782,7 +1783,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
         <v>88</v>
       </c>
@@ -1791,7 +1792,7 @@
       </c>
       <c r="C84" s="2"/>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>89</v>
       </c>
@@ -1802,7 +1803,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>90</v>
       </c>
@@ -1813,7 +1814,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
         <v>91</v>
       </c>
@@ -1824,7 +1825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
         <v>92</v>
       </c>
@@ -1835,7 +1836,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>93</v>
       </c>
@@ -1846,7 +1847,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>94</v>
       </c>
@@ -1857,7 +1858,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
         <v>95</v>
       </c>
@@ -1868,7 +1869,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
         <v>96</v>
       </c>
@@ -1879,7 +1880,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>97</v>
       </c>
@@ -1890,7 +1891,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
         <v>98</v>
       </c>
@@ -1901,7 +1902,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>99</v>
       </c>
@@ -1912,7 +1913,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
         <v>100</v>
       </c>
@@ -1923,7 +1924,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
         <v>101</v>
       </c>
@@ -1934,7 +1935,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
         <v>102</v>
       </c>
@@ -1945,7 +1946,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
         <v>103</v>
       </c>
@@ -1956,7 +1957,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
         <v>104</v>
       </c>
@@ -1967,7 +1968,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
         <v>105</v>
       </c>
@@ -1978,7 +1979,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A102" t="s">
         <v>106</v>
       </c>
@@ -1989,7 +1990,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
         <v>107</v>
       </c>
@@ -2000,7 +2001,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
         <v>108</v>
       </c>
@@ -2011,7 +2012,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A105" t="s">
         <v>109</v>
       </c>
@@ -2022,7 +2023,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A106" t="s">
         <v>110</v>
       </c>
@@ -2033,7 +2034,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
         <v>111</v>
       </c>
@@ -2044,7 +2045,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
         <v>112</v>
       </c>
@@ -2055,7 +2056,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
         <v>113</v>
       </c>
@@ -2066,7 +2067,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A110" t="s">
         <v>114</v>
       </c>
@@ -2077,7 +2078,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A111" t="s">
         <v>115</v>
       </c>
@@ -2088,7 +2089,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
         <v>116</v>
       </c>
@@ -2099,7 +2100,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
         <v>117</v>
       </c>
@@ -2110,7 +2111,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
         <v>118</v>
       </c>
@@ -2121,7 +2122,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
         <v>119</v>
       </c>

</xml_diff>